<commit_message>
Extract S012 and refine scientific RAG novelty
</commit_message>
<xml_diff>
--- a/03-RESEARCH-FOUNDATION/literature_matrix.xlsx
+++ b/03-RESEARCH-FOUNDATION/literature_matrix.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" r:id="R437c949378d74948"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Appraisal" sheetId="2" r:id="Rd38b41746e2d4f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" r:id="R4f02e271f8e04241"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality Appraisal" sheetId="2" r:id="Rf283b5783cea47b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2669,13 +2669,13 @@
         <x:v>S012</x:v>
       </x:c>
       <x:c r="B17" s="31" t="str">
-        <x:v>Title/abstract included</x:v>
+        <x:v>Full text included</x:v>
       </x:c>
       <x:c r="C17" s="31" t="str">
         <x:v>B: RAG and Scientific QA</x:v>
       </x:c>
       <x:c r="D17" s="31" t="str">
-        <x:v>Matos, J., Silva, C., and Goncalo Oliveira, H. (2026). Benchmarking Retrieval-Augmented Generation for Scientific Knowledge QA in European Portuguese. NSLP at LREC 2026, 25-31.</x:v>
+        <x:v>Matos, J., Silva, C., and Gonçalo Oliveira, H. (2026). Benchmarking Retrieval-Augmented Generation for Scientific Knowledge QA in European Portuguese. NSLP at LREC 2026, 25-31.</x:v>
       </x:c>
       <x:c r="E17" s="31" t="str">
         <x:v>https://doi.org/10.63317/3muergicuxwk</x:v>
@@ -2693,71 +2693,85 @@
         <x:v>Empirical method</x:v>
       </x:c>
       <x:c r="J17" s="31" t="str">
-        <x:v>Scientific knowledge question answering</x:v>
+        <x:v>European Portuguese scientific knowledge question answering</x:v>
       </x:c>
       <x:c r="K17" s="31" t="str">
-        <x:v>Measure how retrieval design affects European Portuguese scientific QA with small instruction-tuned models.</x:v>
+        <x:v>Measure how RAG affects scientific multiple-choice QA across open 4-12B instruction-tuned models and retrieval configurations.</x:v>
       </x:c>
       <x:c r="L17" s="31" t="str">
-        <x:v>Portuguese Global MMLU Lite test split and a scientific-literature knowledge base</x:v>
+        <x:v>Portuguese Global MMLU Lite test split and CorEGe-PT scientific knowledge base</x:v>
       </x:c>
       <x:c r="M17" s="33" t="str">
-        <x:v>More than 32,000 scientific documents converted to Markdown</x:v>
+        <x:v>400 Portuguese QA items; more than 32,000 open-access scientific documents</x:v>
       </x:c>
       <x:c r="N17" s="31" t="str">
         <x:v>European Portuguese</x:v>
       </x:c>
       <x:c r="O17" s="31" t="str">
-        <x:v>Scientific text</x:v>
+        <x:v>Scientific text and multiple-choice QA</x:v>
       </x:c>
       <x:c r="P17" s="31" t="str">
-        <x:v>Dense retrieval with multilingual versus Portuguese-specific specialization; k = 1, 3, 5, 10</x:v>
+        <x:v>Dense cosine retrieval; multilingual versus Portuguese-specific encoders; top-30 candidate pool; k = 1, 3, 5, 10</x:v>
       </x:c>
       <x:c r="Q17" s="31" t="str">
-        <x:v>Multilingual and Portuguese-specific retrievers; exact models pending full-text extraction</x:v>
-      </x:c>
-      <x:c r="R17" s="31"/>
+        <x:v>paraphrase-multilingual-mpnet-base-v2 (278M); serafim-335m-portuguese-pt-sentence-encoder-ir (335M)</x:v>
+      </x:c>
+      <x:c r="R17" s="31" t="str">
+        <x:v>Split by Markdown headers, then recursively into 500-character chunks with 50-character overlap</x:v>
+      </x:c>
       <x:c r="S17" s="31" t="str">
-        <x:v>Compared on versus off</x:v>
+        <x:v>gte-multilingual-reranker-base; reranking on versus off</x:v>
       </x:c>
       <x:c r="T17" s="31" t="str">
-        <x:v>Five instruction-tuned small language models (4-12B)</x:v>
-      </x:c>
-      <x:c r="U17" s="31"/>
+        <x:v>AMALIA 9B; EuroLLM-9B-Instruct; Qwen3-8B; Gemma-3-4B-IT; Gemma-3-12B-IT</x:v>
+      </x:c>
+      <x:c r="U17" s="31" t="str">
+        <x:v>None</x:v>
+      </x:c>
       <x:c r="V17" s="31" t="str">
-        <x:v>Language/domain alignment studied rather than Arabic-English transfer</x:v>
-      </x:c>
-      <x:c r="W17" s="31"/>
-      <x:c r="X17" s="31"/>
+        <x:v>No cross-lingual transfer; compares multilingual and Portuguese-specialized retrieval within Portuguese</x:v>
+      </x:c>
+      <x:c r="W17" s="31" t="str">
+        <x:v>None; no generated answer citations</x:v>
+      </x:c>
+      <x:c r="X17" s="31" t="str">
+        <x:v>None; answerability and refusal are not evaluated</x:v>
+      </x:c>
       <x:c r="Y17" s="31" t="str">
-        <x:v>Closed-book baseline and 16 RAG configurations</x:v>
-      </x:c>
-      <x:c r="Z17" s="31"/>
+        <x:v>Closed-book plus 16 RAG configurations per generator</x:v>
+      </x:c>
+      <x:c r="Z17" s="31" t="str">
+        <x:v>No direct chunk-level retrieval metric; downstream task accuracy is used as a proxy</x:v>
+      </x:c>
       <x:c r="AA17" s="31" t="str">
-        <x:v>Scientific QA performance; exact metric definition pending full-text extraction</x:v>
-      </x:c>
-      <x:c r="AB17" s="31"/>
-      <x:c r="AC17" s="31"/>
+        <x:v>Multiple-choice accuracy, standard error, and change from closed-book accuracy</x:v>
+      </x:c>
+      <x:c r="AB17" s="31" t="str">
+        <x:v>Not required for deterministic scoring against gold multiple-choice labels; none reported</x:v>
+      </x:c>
+      <x:c r="AC17" s="31" t="str">
+        <x:v>Two-proportion Z test, McNemar test, and paired subcategory comparisons</x:v>
+      </x:c>
       <x:c r="AD17" s="31" t="str">
-        <x:v>RAG gains were model-dependent; larger k could add retrieval noise, and retriever/reranker language-domain alignment mattered.</x:v>
+        <x:v>RAG effects were generator-dependent. Gemma-3-4B and 12B gained significantly, every Qwen3-8B RAG configuration reduced accuracy, larger k could add noise, and reranking could erase specialized-retriever gains under language/domain mismatch.</x:v>
       </x:c>
       <x:c r="AE17" s="31" t="str">
-        <x:v>European Portuguese rather than Arabic-English; citation and abstention evaluation are not established from the abstract.</x:v>
+        <x:v>Broad multiple-choice benchmark; possible Brazilian Portuguese bias; no direct retrieval evaluation; one chunking strategy; no open-ended generation, citations, faithfulness, abstention, cross-lingual condition, or consumer-hardware evaluation.</x:v>
       </x:c>
       <x:c r="AF17" s="31" t="str">
-        <x:v>Controlled scientific RAG evaluation is needed for other low-resource languages and trustworthiness dimensions.</x:v>
+        <x:v>Open-ended scientific QA, direct grounding evaluation, effective context selection, and language/domain-aligned retrieval pipelines remain open; the Arabic-English claim-level trustworthiness combination is not studied.</x:v>
       </x:c>
       <x:c r="AG17" s="31" t="str">
-        <x:v>Unclear</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="AH17" s="31" t="str">
-        <x:v>Unclear</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="AI17" s="31" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="AJ17" s="31" t="str">
-        <x:v>Direct methodological analogue for small-model scientific RAG; full-text extraction has high priority.</x:v>
+        <x:v>Full-text note: 03-RESEARCH-FOUNDATION/full_text_notes/S012_scientific_rag_ptpt.md</x:v>
       </x:c>
       <x:c r="AK17" s="37" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -5486,7 +5500,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cc3982b0cf044a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64c941dd7b564a25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5893,24 +5907,52 @@
         <x:v>S012</x:v>
       </x:c>
       <x:c r="B17" s="31" t="str">
-        <x:v>Matos, J., Silva, C., and Goncalo Oliveira, H. (2026). Benchmarking Retrieval-Augmented Generation for Scientific Knowledge QA in European Portuguese. NSLP at LREC 2026, 25-31.</x:v>
-      </x:c>
-      <x:c r="C17" s="32"/>
-      <x:c r="D17" s="32"/>
-      <x:c r="E17" s="32"/>
-      <x:c r="F17" s="32"/>
-      <x:c r="G17" s="32"/>
-      <x:c r="H17" s="32"/>
-      <x:c r="I17" s="32"/>
-      <x:c r="J17" s="32"/>
-      <x:c r="K17" s="32"/>
-      <x:c r="L17" s="32"/>
-      <x:c r="M17" s="32"/>
-      <x:c r="N17" s="31"/>
-      <x:c r="O17" s="31"/>
-      <x:c r="P17" s="37"/>
+        <x:v>Matos, J., Silva, C., and Gonçalo Oliveira, H. (2026). Benchmarking Retrieval-Augmented Generation for Scientific Knowledge QA in European Portuguese. NSLP at LREC 2026, 25-31.</x:v>
+      </x:c>
+      <x:c r="C17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G17" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L17" s="32" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M17" s="32" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="N17" s="31" t="str">
+        <x:v>High (provisional)</x:v>
+      </x:c>
+      <x:c r="O17" s="31" t="str">
+        <x:v>AI-assisted extraction; human verification pending</x:v>
+      </x:c>
+      <x:c r="P17" s="37" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="Q17" s="31" t="str">
-        <x:v>Pending full-text appraisal.</x:v>
+        <x:v>Strong controlled factorial evaluation with released code/data, statistical tests, configuration robustness analysis, and explicit limitations. Multiple-choice accuracy is appropriate, but retrieval quality is not evaluated directly. Human evaluation is not required for gold-label option scoring.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
@@ -12728,7 +12770,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61d22bd26714474c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R780a49cbff59454e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>